<commit_message>
Sửa đúng sự thật: nguồn thay đổi v1→v2 là rà soát nội bộ, không phải Chặng 3
Chặng 3 (kiểm tra chéo với nhóm khác) chưa diễn ra. Trước đó memo, README
và dashboard đang diễn đạt CH1-CH4 như "góp ý nhận được từ nhóm bạn" —
sai sự thật, đã sửa lại toàn bộ:

- Sheet 6 dựng lại thành nhật ký đầy đủ 8 thay đổi: CH1-CH4 (Trang, trục
  chỉ số) + CH5-CH8 (Sơn, trục chẩn đoán), cột "Người nêu" ghi rõ từng
  người thay vì để trống "Nhóm phản biện: ______"
- Sheet 1: dòng attribution nói rõ mới qua rà soát nội bộ Chặng 2
- memo §3 và README §6: ghi rõ nguồn nội bộ, liệt kê đủ 8 thay đổi
- Cột "Góp ý đã đưa cho nhóm bạn" trả về trống thật cho cả 3 thành viên

Còn thiếu để đủ §6.5: thay đổi phát sinh từ Chặng 3 thật, sẽ đánh số
từ CH9 và ghi tên nhóm phản biện vào cột "Người nêu".

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -122,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +151,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -530,7 +536,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bản v2 — sau rà soát nội bộ (Chặng 2) và kiểm tra chéo (Chặng 3) · Nhóm Track1badao · Day 28 Track 01. Phân công từng người: xem bảng thành viên ở README. Cột 'Thay đổi so với v1' trên mỗi sheet ghi từng thay đổi; nhật ký đầy đủ ở sheet '6. Thay doi v1 - v2'.</t>
+          <t>Bản v2 — sau rà soát chéo NỘI BỘ trong nhóm (Chặng 2). Kiểm tra chéo với nhóm khác (Chặng 3) CHƯA diễn ra tại thời điểm lập bảng. Nhóm Track1badao · Day 28 Track 01. Phân công từng người: xem bảng thành viên ở README. Cột 'Thay đổi so với v1' trên mỗi sheet ghi từng thay đổi; nhật ký đầy đủ ở sheet '6. Thay doi v1 - v2'.</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1972,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2124,8 +2129,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -2782,58 +2785,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Nhật ký thay đổi sau kiểm tra chéo — v1 → v2</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nhật ký thay đổi v1 → v2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Chặng 3 · Người rà soát và tổng hợp: Lương Thanh Trang (2A202601363). ĐIỀN TÊN NHÓM PHẢN BIỆN vào cột "Nguồn góp ý" trước khi nộp.</t>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>NGUỒN: rà soát chéo NỘI BỘ trong nhóm Track1badao — Chặng 3 (kiểm tra chéo với nhóm khác) chưa diễn ra tại thời điểm lập bảng. Khi Chặng 3 diễn ra, bổ sung từ CH9 trở đi và ghi tên nhóm phản biện vào cột 'Người nêu'. Tổng hợp bảng: Lương Thanh Trang (2A202601363).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Trục phản biện</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Nguồn góp ý</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Góp ý nhận được</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Trục rà soát</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Người nêu</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Vấn đề chỉ ra ở v1</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Thay đổi đã thực hiện ở v2</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Vị trí trong file</t>
         </is>
@@ -2845,14 +2848,14 @@
           <t>CH1</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Chỉ số</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Nhóm phản biện: ______</t>
+          <t>Lương Thanh Trang · rà soát nội bộ</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2877,14 +2880,14 @@
           <t>CH2</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Chỉ số</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Nhóm phản biện: ______</t>
+          <t>Lương Thanh Trang · rà soát nội bộ</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2909,14 +2912,14 @@
           <t>CH3</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Hành động</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Nhóm phản biện: ______</t>
+          <t>Lương Thanh Trang · rà soát nội bộ</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2941,14 +2944,14 @@
           <t>CH4</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Hành động</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Nhóm phản biện: ______</t>
+          <t>Lương Thanh Trang · rà soát nội bộ</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2964,6 +2967,134 @@
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Sheet "4. Lo trinh 30-60-90" · bảng Điều kiện DỪNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CH5</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Chẩn đoán — Gartner-Lite</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Đặng Thái Nam Sơn · rà soát nội bộ</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>v1 chỉ soi Readiness ở nhánh governance. QA mẫu 50 ticket/tuần và hàng đợi ưu tiên SLA 30 phút là CÔNG VIỆC MỚI, chưa giao cho ai và chưa tính vào định biên. Readiness không chỉ là dữ liệu — còn là người và năng lực vận hành thứ mình sắp bật.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Mở Readiness từ 1 lên 4 nhánh, thêm hàng 'Readiness — năng lực vận hành' chấm THIẾU. Gán owner và định biên cho QA mẫu ở bảng kiến trúc tin cậy.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Sheet '2. Chan doan' · bảng 2.2 (hàng mới) · Sheet '3. AS-IS TO-BE' · mắt xích QA mẫu</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CH6</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Chẩn đoán — Gartner-Lite</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Đặng Thái Nam Sơn · rà soát nội bộ</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>v1 chấm Direction ĐẠT. Nhưng cả hệ chỉ số chạy trên baseline giả định: target 70% suy ra từ con số 45% không ai đo. Một hướng đi có đích mà chưa có điểm xuất phát đo được thì chưa kiểm chứng được. Thiếu thêm vế giá trị đặt cạnh chi phí ẩn định kỳ đã nêu ở Day24.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Hạ Direction xuống ĐẠT CÓ ĐIỀU KIỆN, ghi rõ cả hai thiếu sót. Vế giá trị sau đó được lấp bằng M6 (CH2) — hai thay đổi này khép cùng một lỗ hổng.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Sheet '2. Chan doan' · bảng 2.2 · hàng Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CH7</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Chẩn đoán — quan hệ nguyên nhân</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Đặng Thái Nam Sơn · rà soát nội bộ</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>v1 trình bày NN1 và NN2 như hai việc song song. Nhưng TO-BE đòi mỗi đề xuất hoàn tiền kèm tên văn bản · phiên bản · ngày hiệu lực — không thể trích dẫn phiên bản của một tập dữ liệu chưa có trường phiên bản.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Ghi rõ NN1 và NN2 NỐI TIẾP một nửa: nửa NN1 thuộc hội thoại (trích dẫn đoạn chat, mức tin cậy) làm được ngay; nửa thuộc chính sách bị chặn bởi readiness–dữ liệu của NN2. Phiên bản hoá tập chính sách chuyển thành hạng mục bắt buộc của 0–30 ngày và thành điều kiện Gate.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Sheet '2. Chan doan' · kết luận 2.2 và bảng 2.5 · Sheet '4. Lo trinh 30-60-90' · việc chính 0–30 và Gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CH8</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Cách làm mới — vòng học</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Đặng Thái Nam Sơn · rà soát nội bộ</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>v1 nêu vòng phản hồi nhưng không đặt tên nhịp, hiện vật và người chốt — một vòng lặp không có cuộc họp thì không phải vòng lặp. Dữ liệu học lại do chính CSKH sinh ra đúng lúc họ chịu tải cao nhất; không ràng buộc thì nhãn dồn vào 'khác' và vòng học nhận về nhiễu.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Bốn nhãn lý do trả lại thành lựa chọn BẮT BUỘC, 'khác' phải kèm mô tả. Đặt nhịp: họp rà 30 phút mỗi tuần, hiện vật là bảng phân bố loại lỗi, Policy Owner chốt. Thêm kill criteria: 'khác' &gt;15% sau 2 tuần ⇒ nhãn hỏng. Gate 60–90 đòi phân bố loại lỗi dịch chuyển được so với đường cơ sở 100 ca.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Sheet '3. AS-IS TO-BE' · bước 5 và 7 · Sheet '4. Lo trinh 30-60-90' · kill criteria và dấu hiệu 60–90</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rà soát cuối: sửa hai chỗ không nhất quán
- Ghi chú 6 sheet 5 liệt kê M5 vào diện phải hoãn target, nhưng M5 vẫn
  giữ 95%. Sửa ghi chú: M5 là ngoại lệ có lý do — 95% là cam kết SLA do
  tổ chức tự đặt, không phải mức cải thiện suy ra từ baseline
- Đổi "chờ Chặng 3" thành "không tham gia Chặng 3" và nói rõ lý do cột 4
  trống, thay vì để ngỏ như thể sắp có

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -540,7 +540,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1973,7 +1972,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2131,8 +2129,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -2335,6 +2331,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -2806,6 +2804,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -2851,7 +2850,7 @@
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>6. (v2) KHÔNG đặt target dạng phần trăm cụ thể trên một baseline ghi 'chưa đo' (M5, M6, M7). Target của ba chỉ số này chỉ được chốt sau giai đoạn 0–30 ngày. Đặt trước là lặp đúng lỗi đã bắt ở CH6 khi hạ Direction.</t>
+          <t>6. (v2) KHÔNG đặt target dạng phần trăm cụ thể trên một baseline ghi 'chưa đo' — áp cho M6 và M7; target của hai chỉ số này chỉ chốt sau giai đoạn 0–30 ngày. Đặt trước là lặp đúng lỗi đã bắt ở CH6 khi hạ Direction. M5 là ngoại lệ có lý do: 95% là một CAM KẾT SLA do tổ chức tự đặt ra, không phải mức cải thiện suy ra từ hiện trạng — loại target này không cần baseline mới đặt được.</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2906,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>